<commit_message>
update case of population density study
</commit_message>
<xml_diff>
--- a/Case of population density study/Case of population density study.xlsx
+++ b/Case of population density study/Case of population density study.xlsx
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.7538775510204082</v>
+        <v>0.574825</v>
       </c>
       <c r="D2">
-        <v>1.11097546412554E-19</v>
+        <v>0.01953434099771332</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.1976190476190476</v>
+        <v>0.0892</v>
       </c>
       <c r="D3">
-        <v>4.543831970400404E-35</v>
+        <v>3.830104392717387E-116</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +427,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.8355328798185941</v>
+        <v>0.267125</v>
       </c>
       <c r="D4">
-        <v>9.586181619044839E-44</v>
+        <v>8.221766729351771E-16</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.2065986394557823</v>
+        <v>0.07675</v>
       </c>
       <c r="D5">
-        <v>6.101270598773862E-32</v>
+        <v>6.249809659430056E-148</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.6279365079365079</v>
+        <v>0.224575</v>
       </c>
       <c r="D6">
-        <v>4.342087764136911E-05</v>
+        <v>1.628640956960896E-23</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.5094784580498867</v>
+        <v>0.47705</v>
       </c>
       <c r="D7">
-        <v>0.7677154773804721</v>
+        <v>0.4880176104578198</v>
       </c>
     </row>
   </sheetData>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.6994707974253584</v>
+        <v>0.7291112340047301</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.2869663329224457</v>
+        <v>0.4049899717392053</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.6995846536086174</v>
+        <v>0.7242901714077284</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -585,10 +585,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.04546301856080344</v>
+        <v>0.4292317231265865</v>
       </c>
       <c r="D5">
-        <v>0.01602150947374636</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.8974127457079115</v>
+        <v>0.916775182465226</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.8626915483608316</v>
+        <v>0.927998976252987</v>
       </c>
       <c r="D7">
         <v>0</v>

</xml_diff>

<commit_message>
re-execute case study 2
</commit_message>
<xml_diff>
--- a/Case of population density study/Case of population density study.xlsx
+++ b/Case of population density study/Case of population density study.xlsx
@@ -10,7 +10,8 @@
     <sheet name="gcmc" sheetId="1" r:id="rId1"/>
     <sheet name="gccm" sheetId="2" r:id="rId2"/>
     <sheet name="pcc" sheetId="3" r:id="rId3"/>
-    <sheet name="gd" sheetId="4" r:id="rId4"/>
+    <sheet name="directlingam" sheetId="4" r:id="rId4"/>
+    <sheet name="gd" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -391,10 +392,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.5754</v>
+        <v>0.6186578798185941</v>
       </c>
       <c r="D2">
-        <v>0.01861243455681576</v>
+        <v>0.0006192749108928587</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +410,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.08985</v>
+        <v>0.1063633786848073</v>
       </c>
       <c r="D3">
-        <v>5.082649054564429E-115</v>
+        <v>2.155995784578711E-74</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +428,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.2675</v>
+        <v>0.3006306689342403</v>
       </c>
       <c r="D4">
-        <v>9.449794499962948E-16</v>
+        <v>1.757118450130801E-09</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +446,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.077025</v>
+        <v>0.09279336734693877</v>
       </c>
       <c r="D5">
-        <v>2.308728324280074E-147</v>
+        <v>7.74111461817066E-95</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +464,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.224925</v>
+        <v>0.2424178004535147</v>
       </c>
       <c r="D6">
-        <v>1.985033547688675E-23</v>
+        <v>1.674870268848038E-16</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +482,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.4775</v>
+        <v>0.5001771541950113</v>
       </c>
       <c r="D7">
-        <v>0.4965603480241145</v>
+        <v>0.9961253644644774</v>
       </c>
     </row>
   </sheetData>
@@ -531,7 +532,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.7291112340047301</v>
+        <v>0.7291112340047295</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -549,7 +550,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.4049899717392053</v>
+        <v>0.4049899717392104</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -567,7 +568,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.7242901714077284</v>
+        <v>0.7242901714077293</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -585,7 +586,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.4292317231265865</v>
+        <v>0.4292317231265871</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -603,7 +604,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.916775182465226</v>
+        <v>0.9167751824652264</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -621,7 +622,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.927998976252987</v>
+        <v>0.9279989762529879</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -662,12 +663,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>popd</t>
+          <t>elev</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>elev</t>
+          <t>popd</t>
         </is>
       </c>
       <c r="C2">
@@ -680,12 +681,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>popd</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>popd</t>
         </is>
       </c>
       <c r="C3">
@@ -698,12 +699,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>elev</t>
+          <t>popd</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>popd</t>
+          <t>elev</t>
         </is>
       </c>
       <c r="C4">
@@ -716,12 +717,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>elev</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>elev</t>
         </is>
       </c>
       <c r="C5">
@@ -734,12 +735,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>popd</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>popd</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="C6">
@@ -752,12 +753,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>elev</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>elev</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="C7">
@@ -802,6 +803,146 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>elev</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>popd</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>popd</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1.631331429283576E-155</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>popd</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>elev</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>-0.06312474262787934</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>elev</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>5.881623579974856E-178</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>popd</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>9.452529659072905E-05</v>
+      </c>
+      <c r="D6">
+        <v>1.631331429283576E-155</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>elev</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>-0.003174165728771098</v>
+      </c>
+      <c r="D7">
+        <v>5.881623579974856E-178</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>cause</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>effect</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cs</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>tem</t>
         </is>
       </c>

</xml_diff>